<commit_message>
Expand directory: add Discord, LinkedIn & CSM sections + browser version
- Add Discord, LinkedIn and a cross-platform Customer/Client Success
  Manager (CSM) section to the spreadsheet (85 communities total).
- Add self-contained, searchable browser version (high_ticket_directory.html)
  with platform + job/general filters and live text search.
- Consolidate data into a single generator (build.py) that emits both the
  xlsx and the html from one source of truth.

https://claude.ai/code/session_01GUJ8qSByy4U4SPUEowsMsA
</commit_message>
<xml_diff>
--- a/High_Ticket_Sales_Groups.xlsx
+++ b/High_Ticket_Sales_Groups.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="High Ticket Sales Groups" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="High Ticket Groups" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +49,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -58,7 +58,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="001877F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,6 +69,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB800"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005865F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A66C2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0034A853"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,17 +118,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -117,6 +135,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -486,12 +516,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -505,7 +535,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Job-specific  (job boards / closer &amp; setter opportunities)</t>
+          <t>Job-specific - job boards / closer &amp; setter opportunities</t>
         </is>
       </c>
     </row>
@@ -539,7 +569,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Active job board for high-ticket closing &amp; appointment-setting roles; posts 2-3 times daily plus advice and events.</t>
+          <t>Active job board for high-ticket closing &amp; appointment-setting roles; posts 2-3x daily plus advice and events.</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -561,7 +591,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Dan Lok's members-only community for graduates/closers – networking, opportunities and high-ticket closing support.</t>
+          <t>Dan Lok's members-only community for graduates/closers - networking, opportunities and high-ticket closing support.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -732,12 +762,12 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Matt's Remote Setters &amp; Closers Network (High Ticket)</t>
+          <t>High Ticket Closing: Sales Jobs For Setters &amp; Closers</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Network posting remote high-ticket setter &amp; closer roles plus a linked free Skool/cash competition.</t>
+          <t>Job board for high-ticket setter and closer roles.</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -747,19 +777,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/highticketcloserss/</t>
+          <t>https://www.facebook.com/groups/highticketsalesjobsforclosersandsetters/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Appointment Setters and Closers</t>
+          <t>Matt's Remote Setters &amp; Closers Network (High Ticket)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Opportunity group for high-ticket appointment setters and closers.</t>
+          <t>Network posting remote high-ticket setter &amp; closer roles plus a linked free Skool/cash competition.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -769,19 +799,19 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/267330199599984/</t>
+          <t>https://www.facebook.com/groups/highticketcloserss/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Appointment Setting | Closers &amp; Sales Rep (Impact Closers)</t>
+          <t>High Ticket Appointment Setters and Closers</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Job and opportunity board for high-ticket appointment setters, closers and sales reps.</t>
+          <t>Opportunity group for high-ticket appointment setters and closers.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -791,19 +821,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/impactclosers/</t>
+          <t>https://www.facebook.com/groups/267330199599984/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Titans (Setters/Closers Opportunities)</t>
+          <t>High Ticket Appointment Setting | Closers &amp; Sales Rep (Impact Closers)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Opportunities and resources for high-ticket appointment setters and closers.</t>
+          <t>Job and opportunity board for high-ticket appointment setters, closers and sales reps.</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -813,19 +843,19 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/1601202083962570/</t>
+          <t>https://www.facebook.com/groups/impactclosers/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>CANADIAN JOBS - Appointment Setters &amp; Sales Closers</t>
+          <t>High Ticket Titans (Setters/Closers Opportunities)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Canada-focused job board for appointment setters and sales closers.</t>
+          <t>Opportunities and resources for high-ticket appointment setters and closers.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -835,19 +865,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/327324528755233/</t>
+          <t>https://www.facebook.com/groups/1601202083962570/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales / Remote Closers - AUSTRALIAN</t>
+          <t>High Ticket SMMA / Appointment Setting &amp; Closing 💰</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Australia-focused group for high-ticket sales and remote closing roles.</t>
+          <t>Group for SMMA owners and high-ticket setters/closers - opportunities and tactics.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -857,114 +887,114 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/3470780863202640/</t>
+          <t>https://www.facebook.com/groups/702508090786804/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>CANADIAN JOBS - Appointment Setters &amp; Sales Closers</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Canada-focused job board for appointment setters and sales closers.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/327324528755233/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales / Remote Closers - AUSTRALIAN</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Australia-focused group for high-ticket sales and remote closing roles.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/3470780863202640/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Setter y Closer HIGH TICKET LATINOAMERICA</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Spanish-language Latin-America group for high-ticket setters and closers.</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/settersyclosershighticket/</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>General  (training, networking &amp; community)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>General - training, networking &amp; community</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>High-Ticket Sales - ELITE Community For Closers</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Community for closers focused on high-ticket sales skills, training and networking.</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/eliteclosers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>The Closers Dojo - High Ticket Sales Training &amp; Job Opportunities</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Free remote high-ticket sales training plus job opportunities (Kris Cochrane).</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/theclosersdojo/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>High-Ticket Closers | Remote Sales Opportunities &amp; Training (The Advancing Mind)</t>
+          <t>High-Ticket Sales - ELITE Community For Closers</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Blends remote sales opportunities with high-ticket closing training and mindset content.</t>
+          <t>Community for closers focused on high-ticket sales skills, training and networking.</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -974,19 +1004,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/theadvancingmind/</t>
+          <t>https://www.facebook.com/groups/eliteclosers/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Sales People, High Ticket Closers &amp; Setters Community</t>
+          <t>The Closers Dojo - High Ticket Sales Training &amp; Job Opportunities</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>General community for salespeople, high-ticket closers and setters to learn and connect.</t>
+          <t>Free remote high-ticket sales training plus job opportunities (Kris Cochrane).</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -996,19 +1026,19 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/salespeopleandclosers/</t>
+          <t>https://www.facebook.com/groups/theclosersdojo/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>The Elite-Closers Community</t>
+          <t>High-Ticket Closers | Remote Sales Opportunities &amp; Training (The Advancing Mind)</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Community for elite closers sharing high-ticket sales strategy and support.</t>
+          <t>Blends remote sales opportunities with high-ticket closing training and mindset content.</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1018,19 +1048,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/elitesalesclosers/</t>
+          <t>https://www.facebook.com/groups/theadvancingmind/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Club Closer Community | High Ticket Sales and Closers</t>
+          <t>Sales People, High Ticket Closers &amp; Setters Community</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Community hub for high-ticket sales and closers.</t>
+          <t>General community for salespeople, high-ticket closers and setters to learn and connect.</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -1040,19 +1070,19 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/823218068832896/</t>
+          <t>https://www.facebook.com/groups/salespeopleandclosers/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>The Closers Community</t>
+          <t>The Elite-Closers Community</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>General community for closers around high-ticket sales.</t>
+          <t>Community for elite closers sharing high-ticket sales strategy and support.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -1062,19 +1092,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/thecloserscom/</t>
+          <t>https://www.facebook.com/groups/elitesalesclosers/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Remote Closing Academy (Cole Gordon - private group)</t>
+          <t>Club Closer Community | High Ticket Sales and Closers</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Private student community for Cole Gordon's Remote Closing Academy: training, livestreams and peer feedback.</t>
+          <t>Community hub for high-ticket sales and closers.</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -1084,143 +1114,143 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/1754793088033322/</t>
+          <t>https://www.facebook.com/groups/823218068832896/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
+          <t>The Closers Community</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>General community for closers around high-ticket sales.</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/thecloserscom/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Remote Closing Academy (Cole Gordon - private group)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Private student community for Cole Gordon's Remote Closing Academy: training, livestreams and peer feedback.</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1754793088033322/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
           <t>Closer Babes - Remote High-Ticket Sales Training for Women</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Women-focused remote high-ticket sales training and community (group accessed via the program site).</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Via program site</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>https://closerbabes.com/</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>SKOOL</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Job-specific  (recruitment, placement &amp; hiring marketplaces)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Job-specific - recruitment, placement &amp; hiring marketplaces</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Remote Closing Community (RCC)</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Members-only marketplace connecting setters/closers with founders hiring; screened job posts every 24-48h. 7-day free trial then $27/mo.</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>~1,000+</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/remote-closing-community-5761/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>ORA - High Ticket Recruitment</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Free training + recruitment connecting 7-9 figure businesses with elite remote closers, setters and managers.</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/free-high-ticket-sales-recruit-3019/about</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Sales Training &amp; Placement (The Sales Agency)</t>
+          <t>Remote Closing Community (RCC)</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Robb Quinn's community: closer's playbook, weekly war-room calls and priority access to elite remote sales roles.</t>
+          <t>Members-only marketplace connecting setters/closers with founders hiring; screened job posts every 24-48h. 7-day free trial then $27/mo.</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Login required</t>
+          <t>~1,000+</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/thesalesagency/about</t>
+          <t>https://www.skool.com/remote-closing-community-5761/about</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Remote Sales Placement (The High Ticket Bridge)</t>
+          <t>ORA - High Ticket Recruitment</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Trains and places high-ticket closers into remote sales roles.</t>
+          <t>Free training + recruitment connecting 7-9 figure businesses with elite remote closers, setters and managers.</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1230,19 +1260,19 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/the-high-ticket-bridge/about</t>
+          <t>https://www.skool.com/free-high-ticket-sales-recruit-3019/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales | BOC™</t>
+          <t>Sales Training &amp; Placement (The Sales Agency)</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Free high-ticket sales network to hire and get hired into appointment-setting and closing roles.</t>
+          <t>Robb Quinn's community: closer's playbook, weekly war-room calls and priority access to elite remote sales roles.</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -1252,19 +1282,19 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/appointmentsetters/about</t>
+          <t>https://www.skool.com/thesalesagency/about</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Setter™</t>
+          <t>Remote Sales Placement (The High Ticket Bridge)</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Positions itself as the #1 community training and creating top high-ticket appointment setters.</t>
+          <t>Trains and places high-ticket closers into remote sales roles.</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -1274,19 +1304,19 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-setter-7793/about</t>
+          <t>https://www.skool.com/the-high-ticket-bridge/about</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Titans</t>
+          <t>High Ticket Sales | BOC™</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>For appointment setters who want to perfect their skills and land jobs at top companies in their niche.</t>
+          <t>Free high-ticket sales network to hire and get hired into appointment-setting and closing roles.</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -1296,19 +1326,19 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-titans-3792/about</t>
+          <t>https://www.skool.com/appointmentsetters/about</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Superior Setters</t>
+          <t>High Ticket Setter™</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Community of remote-sales setters learning to become A-game appointment setters.</t>
+          <t>Positions itself as the #1 community training and creating top high-ticket appointment setters.</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -1318,19 +1348,19 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/superior-setters-1902/about</t>
+          <t>https://www.skool.com/high-ticket-setter-7793/about</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Appointment Setter (Free)</t>
+          <t>High Ticket Titans</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Coaching community (1,200+ setters coached) to book calls and land high-ticket opportunities.</t>
+          <t>For appointment setters who want to perfect their skills and land jobs at top companies in their niche.</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -1340,19 +1370,19 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/appointmentsetting/about</t>
+          <t>https://www.skool.com/high-ticket-titans-3792/about</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Sales Community for Closers</t>
+          <t>Superior Setters</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Community that regularly posts remote high-ticket closer roles with top commissions.</t>
+          <t>Community of remote-sales setters learning to become A-game appointment setters.</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -1362,19 +1392,19 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/sales-community-for-closers-1459</t>
+          <t>https://www.skool.com/superior-setters-1902/about</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Elite Closers</t>
+          <t>Appointment Setter (Free)</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Closer community that posts active high-ticket sales hiring ($5-8K/mo OTE roles).</t>
+          <t>Coaching community (1,200+ setters coached) to book calls and land high-ticket opportunities.</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -1384,19 +1414,19 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/eliteclosers</t>
+          <t>https://www.skool.com/appointmentsetting/about</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Staffing World</t>
+          <t>Closers Inner Circle (Job Opportunities)</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Staffing/agency community recruiting remote high-ticket closers.</t>
+          <t>Closer community posting remote high-ticket job opportunities.</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -1406,19 +1436,19 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/agencyworld</t>
+          <t>https://www.skool.com/closers-circle/about</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Elite Remote Closers Network</t>
+          <t>Sales Community for Closers</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Network for remote high-ticket closers with opportunities and frank industry guidance.</t>
+          <t>Community that regularly posts remote high-ticket closer roles with top commissions.</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -1428,180 +1458,180 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/elite-remote-closers-network-3228</t>
+          <t>https://www.skool.com/sales-community-for-closers-1459</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Setter To Closer - Elite</t>
+          <t>Elite Closers</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Community focused on progressing setters into closing roles.</t>
+          <t>Closer community that posts active high-ticket sales hiring ($5-8K/mo OTE roles).</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>~78</t>
+          <t>Login required</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/setter-to-closer-elite-3793/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>General  (training, mastermind &amp; community)</t>
+          <t>https://www.skool.com/eliteclosers</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Staffing World</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Staffing/agency community recruiting remote high-ticket closers.</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/agencyworld</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Elite Remote Closers Network</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Network for remote high-ticket closers with opportunities and frank industry guidance.</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/elite-remote-closers-network-3228</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Group / Community</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>What it's advertised as</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Members</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Remote Sales Job Accelerator</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Teaches how to land a remote sales role paying $4-10k/mo with no prior experience.</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remotesalesjobaccelerator/about</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>High-Ticket Sales Society</t>
+          <t>Setter To Closer - Elite</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Free community (Chris Campbell) for mastering sales, marketing &amp; mindset; learn to earn $10k-$25k+/mo as a remote closer.</t>
+          <t>Community focused on progressing setters into closing roles.</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>~2,200</t>
+          <t>~78</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-sales/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Force</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Community for closers, setters &amp; online businesses focused on hiring, coaching, leadership and scaling revenue.</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/high-ticket-force-3713/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Skool for High Ticket Sales (High Ticket Millions)</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>For experts who've sold $10k+ of their own offers; win higher-paying clients and recurring revenue via Skool.</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/high-ticket-millions-6222/about</t>
+          <t>https://www.skool.com/setter-to-closer-elite-3793/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>General - training, mastermind &amp; community</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Blueprint</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>Mission-driven community empowering high-ticket closers to master sales, accountability and financial freedom.</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/traveling-sales-team-9554</t>
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Training</t>
+          <t>High-Ticket Sales Society</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Free group for high-ticket setters and closers looking to reach their A-player potential.</t>
+          <t>Free community (Chris Campbell) for mastering sales, marketing &amp; mindset; learn to earn $10k-$25k+/mo as a remote closer.</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Login required</t>
+          <t>~2,200</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-sales-training/about</t>
+          <t>https://www.skool.com/high-ticket-sales/about</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Battle</t>
+          <t>High Ticket Force</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Free group for remote salespeople wanting to fast-track into remote high-ticket sales from home.</t>
+          <t>Community for closers, setters &amp; online businesses focused on hiring, coaching, leadership and scaling revenue.</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -1611,19 +1641,19 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-sales-battle</t>
+          <t>https://www.skool.com/high-ticket-force-3713/about</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>The Serial Sales Community</t>
+          <t>Skool for High Ticket Sales (High Ticket Millions)</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket sales skills and growth.</t>
+          <t>For experts who've sold $10k+ of their own offers; win higher-paying clients and recurring revenue via Skool.</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -1633,19 +1663,19 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/serialsales/about</t>
+          <t>https://www.skool.com/high-ticket-millions-6222/about</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Remote Closing Bootcamp</t>
+          <t>High Ticket Sales Blueprint</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Free community to break into remote high-ticket sales – where to find offers and the fundamentals of closing.</t>
+          <t>Mission-driven community empowering high-ticket closers to master sales, accountability and financial freedom.</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -1655,19 +1685,19 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/closing-authority-saless/about</t>
+          <t>https://www.skool.com/traveling-sales-team-9554</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>XCloser.com (Remote Closing)</t>
+          <t>High Ticket Sales Training</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Free remote-sales community with 101 coaching calls on your setter/closer journey.</t>
+          <t>Free group for high-ticket setters and closers looking to reach their A-player potential.</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -1677,19 +1707,19 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/xclosercom-free-training-3117</t>
+          <t>https://www.skool.com/high-ticket-sales-training/about</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>The Closers Academy</t>
+          <t>High Ticket Sales Battle</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Mastermind for ambitious remote high-ticket closers, coaches and experts (CTA system).</t>
+          <t>Free group for remote salespeople wanting to fast-track into remote high-ticket sales from home.</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -1699,19 +1729,19 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/theclosersacademy/about</t>
+          <t>https://www.skool.com/high-ticket-sales-battle</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales University (Remote Closer Mastery)</t>
+          <t>The High Ticket Sales Academy (Psychological Sales)</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Training community for remote high-ticket closing skills.</t>
+          <t>Sales-skills community focused on the psychology of closing high-ticket offers.</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -1721,19 +1751,19 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remote-closer-mastery-3732/about</t>
+          <t>https://www.skool.com/psychological-sales</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>The Remote Closing Lab</t>
+          <t>The Serial Sales Community</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Serves remote high-ticket closers, SDRs and setters with coaching, recruitment and accountability.</t>
+          <t>General sales community covering high-ticket sales skills and growth.</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
@@ -1743,19 +1773,19 @@
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remoteclosinglab/about</t>
+          <t>https://www.skool.com/serialsales/about</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Quantum Sales Academy™</t>
+          <t>Remote Closing Bootcamp</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Sales academy community training remote high-ticket closers (also posts roles).</t>
+          <t>Free community to break into remote high-ticket sales - where to find offers and the fundamentals of closing.</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -1765,19 +1795,19 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/qsa</t>
+          <t>https://www.skool.com/closing-authority-saless/about</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Sales Genius University</t>
+          <t>XCloser.com (Remote Closing)</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Training community running webinars on breaking into remote high-ticket sales.</t>
+          <t>Free remote-sales community with 101 coaching calls on your setter/closer journey.</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -1787,19 +1817,19 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/salesgeniuses</t>
+          <t>https://www.skool.com/xclosercom-free-training-3117</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Remote Closing Club</t>
+          <t>The Closers Academy</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Community for remote closers focused on high-ticket sales skills.</t>
+          <t>Mastermind for ambitious remote high-ticket closers, coaches and experts (CTA system).</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -1809,48 +1839,908 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remote-closing-club-4755/about</t>
+          <t>https://www.skool.com/theclosersacademy/about</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Sales University (Remote Closer Mastery)</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Training community for remote high-ticket closing skills.</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remote-closer-mastery-3732/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>The Remote Closing Lab</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Serves remote high-ticket closers, SDRs and setters with coaching, recruitment and accountability.</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remoteclosinglab/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>Quantum Sales Academy™</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Sales academy community training remote high-ticket closers (also posts roles).</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/qsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Sales Genius University</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Training community running webinars on breaking into remote high-ticket sales.</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/salesgeniuses</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>Remote Closing Club</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Community for remote closers focused on high-ticket sales skills.</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remote-closing-club-4755/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
           <t>High Ticket Closers</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>General high-ticket closer community on Skool.</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/high-ticket-closers-4841/about</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="48" customHeight="1">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>Notes: Member counts shown are those publicly visible at time of research (12 Jun 2026). 'Login required' = the group/Skool page hides its count behind a login, so a number could not be verified without joining. Counts and links change frequently – verify before outreach. Many of these are marketing/lead-gen communities for paid programs.</t>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>DISCORD</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Job-specific - offer placement / job &amp; lead boards</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>High Flow Closers / FlowClose</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>https://top.gg/discord/servers/766313238700785664</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales Closers</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/highticketsalesclosers</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Appointment Setter Life</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/appsetterlife</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Appointment Setter Jobs</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>DISBOARD-listed server functioning as an appointment-setter job board.</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>https://disboard.org/server/1332654195958087681</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>General - training, networking &amp; community</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Prosper</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>TheCloserCommunity</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/8qxyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales Rep</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/highticketsalesrep</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>Sales Pros</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>General sales community covering high-ticket closing skills and networking.</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/salespros</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>DISBOARD - 'high-ticket-sales' tag (directory)</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Browse/discovery page listing many high-ticket-sales Discord servers, sorted by activity.</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="26" customHeight="1">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>LINKEDIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Job-specific - recruiters / pages posting high-ticket roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>Elite Closers (company page)</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/eliteclosers</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Closer Club</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Jobs - 'high ticket closer / setter'</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn job-search feed where agencies (WFS Group, 1 Call Closers, Grant Cardone Enterprises, etc.) post high-ticket roles.</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>N/A (job board)</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=high%20ticket%20closer</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>General - training pages &amp; professional community</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales Academy</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Company page sharing high-ticket sales professional-development content and community.</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>Note on LinkedIn Groups</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn has largely sunset native 'Groups' for this niche - presence now lives in company pages, hashtags (#highticketsales, #remoteclosing) and the jobs feed.</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr"/>
+    </row>
+    <row r="103" ht="26" customHeight="1">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>CUSTOMER SUCCESS / CLIENT SUCCESS MANAGER (CSM) - ALL PLATFORMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Job-specific - high-ticket / remote CSM training &amp; placement</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/client-success/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Client Success Club (alt)  [Skool]</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/client-success-club/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/648104543815634/</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Virtual Assistant - Job Offers board  [Skool]</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Active job board that regularly posts remote Client/Customer Success Manager openings alongside VA roles.</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/virtual-assistant-8842</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>General - customer-success professional communities</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>Group / Community</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>What it's advertised as</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>Customer Success Collective  [LinkedIn + Slack]</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>10,000+ (Slack)</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>https://customersuccess.network/</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>~65,000+</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>https://www.customersuccessassociation.com/forum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Customer Success Leadership Network  [LinkedIn]</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>~14,300 followers</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Gain Grow Retain  [Slack/Web]</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>https://gaingrowretain.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>CS Cafe  [Slack]</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thecscafe.com/p/community</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Customer Success Network (CSM Practice)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence of the CS community - templates, videos, reviews and event announcements.</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/customersuccessnetwork</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="70" customHeight="1">
+      <c r="A121" s="11" t="inlineStr">
+        <is>
+          <t>Notes: Member counts shown are those publicly visible at time of research (12 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="16">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A103:D103"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A104:D104"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A111:D111"/>
+    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="A98:D98"/>
+    <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId1"/>
@@ -1869,8 +2759,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId21"/>
@@ -1878,8 +2768,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId30"/>
@@ -1892,10 +2782,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId46"/>
@@ -1908,6 +2798,35 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh Communities: add 3 new Skool communities (88 total), update research date to 16 Jun 2026
</commit_message>
<xml_diff>
--- a/High_Ticket_Sales_Groups.xlsx
+++ b/High_Ticket_Sales_Groups.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1572,88 +1572,88 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Remote Sales Secrets - Job Board</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Skool community running a remote-sales job board for setters and closers breaking into high-ticket roles.</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remote-sales-secrets</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>General - training, mastermind &amp; community</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>High-Ticket Sales Society</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Free community (Chris Campbell) for mastering sales, marketing &amp; mindset; learn to earn $10k-$25k+/mo as a remote closer.</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>~2,200</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/high-ticket-sales/about</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Force</t>
+          <t>High-Ticket Sales Society</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Community for closers, setters &amp; online businesses focused on hiring, coaching, leadership and scaling revenue.</t>
+          <t>Free community (Chris Campbell) for mastering sales, marketing &amp; mindset; learn to earn $10k-$25k+/mo as a remote closer.</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Login required</t>
+          <t>~2,200</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-force-3713/about</t>
+          <t>https://www.skool.com/high-ticket-sales/about</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Skool for High Ticket Sales (High Ticket Millions)</t>
+          <t>High Ticket Force</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>For experts who've sold $10k+ of their own offers; win higher-paying clients and recurring revenue via Skool.</t>
+          <t>Community for closers, setters &amp; online businesses focused on hiring, coaching, leadership and scaling revenue.</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -1663,19 +1663,19 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-millions-6222/about</t>
+          <t>https://www.skool.com/high-ticket-force-3713/about</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Blueprint</t>
+          <t>Skool for High Ticket Sales (High Ticket Millions)</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Mission-driven community empowering high-ticket closers to master sales, accountability and financial freedom.</t>
+          <t>For experts who've sold $10k+ of their own offers; win higher-paying clients and recurring revenue via Skool.</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -1685,19 +1685,19 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/traveling-sales-team-9554</t>
+          <t>https://www.skool.com/high-ticket-millions-6222/about</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Training</t>
+          <t>High Ticket Sales Blueprint</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Free group for high-ticket setters and closers looking to reach their A-player potential.</t>
+          <t>Mission-driven community empowering high-ticket closers to master sales, accountability and financial freedom.</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -1707,19 +1707,19 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-sales-training/about</t>
+          <t>https://www.skool.com/traveling-sales-team-9554</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Battle</t>
+          <t>High Ticket Sales Training</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Free group for remote salespeople wanting to fast-track into remote high-ticket sales from home.</t>
+          <t>Free group for high-ticket setters and closers looking to reach their A-player potential.</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/high-ticket-sales-battle</t>
+          <t>https://www.skool.com/high-ticket-sales-training/about</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>The High Ticket Sales Academy (Psychological Sales)</t>
+          <t>High Ticket Sales Battle</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Sales-skills community focused on the psychology of closing high-ticket offers.</t>
+          <t>Free group for remote salespeople wanting to fast-track into remote high-ticket sales from home.</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -1751,19 +1751,19 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/psychological-sales</t>
+          <t>https://www.skool.com/high-ticket-sales-battle</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>The Serial Sales Community</t>
+          <t>The High Ticket Sales Academy (Psychological Sales)</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket sales skills and growth.</t>
+          <t>Sales-skills community focused on the psychology of closing high-ticket offers.</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
@@ -1773,19 +1773,19 @@
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/serialsales/about</t>
+          <t>https://www.skool.com/psychological-sales</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Remote Closing Bootcamp</t>
+          <t>The Serial Sales Community</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Free community to break into remote high-ticket sales - where to find offers and the fundamentals of closing.</t>
+          <t>General sales community covering high-ticket sales skills and growth.</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -1795,19 +1795,19 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/closing-authority-saless/about</t>
+          <t>https://www.skool.com/serialsales/about</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>XCloser.com (Remote Closing)</t>
+          <t>Remote Closing Bootcamp</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Free remote-sales community with 101 coaching calls on your setter/closer journey.</t>
+          <t>Free community to break into remote high-ticket sales - where to find offers and the fundamentals of closing.</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -1817,19 +1817,19 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/xclosercom-free-training-3117</t>
+          <t>https://www.skool.com/closing-authority-saless/about</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>The Closers Academy</t>
+          <t>XCloser.com (Remote Closing)</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Mastermind for ambitious remote high-ticket closers, coaches and experts (CTA system).</t>
+          <t>Free remote-sales community with 101 coaching calls on your setter/closer journey.</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -1839,19 +1839,19 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/theclosersacademy/about</t>
+          <t>https://www.skool.com/xclosercom-free-training-3117</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales University (Remote Closer Mastery)</t>
+          <t>The Closers Academy</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Training community for remote high-ticket closing skills.</t>
+          <t>Mastermind for ambitious remote high-ticket closers, coaches and experts (CTA system).</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -1861,19 +1861,19 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remote-closer-mastery-3732/about</t>
+          <t>https://www.skool.com/theclosersacademy/about</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>The Remote Closing Lab</t>
+          <t>High Ticket Sales University (Remote Closer Mastery)</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Serves remote high-ticket closers, SDRs and setters with coaching, recruitment and accountability.</t>
+          <t>Training community for remote high-ticket closing skills.</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -1883,19 +1883,19 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remoteclosinglab/about</t>
+          <t>https://www.skool.com/remote-closer-mastery-3732/about</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Quantum Sales Academy™</t>
+          <t>The Remote Closing Lab</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Sales academy community training remote high-ticket closers (also posts roles).</t>
+          <t>Serves remote high-ticket closers, SDRs and setters with coaching, recruitment and accountability.</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -1905,19 +1905,19 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/qsa</t>
+          <t>https://www.skool.com/remoteclosinglab/about</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Sales Genius University</t>
+          <t>Quantum Sales Academy™</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Training community running webinars on breaking into remote high-ticket sales.</t>
+          <t>Sales academy community training remote high-ticket closers (also posts roles).</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -1927,19 +1927,19 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/salesgeniuses</t>
+          <t>https://www.skool.com/qsa</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Remote Closing Club</t>
+          <t>Sales Genius University</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Community for remote closers focused on high-ticket sales skills.</t>
+          <t>Training community running webinars on breaking into remote high-ticket sales.</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -1949,260 +1949,260 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/remote-closing-club-4755/about</t>
+          <t>https://www.skool.com/salesgeniuses</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
+          <t>Remote Closing Club</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Community for remote closers focused on high-ticket sales skills.</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/remote-closing-club-4755/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
           <t>High Ticket Closers</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>General high-ticket closer community on Skool.</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/high-ticket-closers-4841/about</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="8" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Sales Elites</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Community for closers, setters and ambitious salespeople mastering high-ticket sales — with opportunities posted by members actively building sales teams.</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/saleselites/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>6Figure Appointment Setter (Next Level Closers)</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Training community helping appointment setters level up into six-figure remote setting and closing roles.</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/next-level-closers-4020</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>DISCORD</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Job-specific - offer placement / job &amp; lead boards</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>High Flow Closers / FlowClose</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>https://top.gg/discord/servers/766313238700785664</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Closers</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>https://discord.me/highticketsalesclosers</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>Appointment Setter Life</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>https://discord.me/appsetterlife</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
+          <t>High Flow Closers / FlowClose</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>https://top.gg/discord/servers/766313238700785664</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales Closers</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/highticketsalesclosers</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Appointment Setter Life</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/appsetterlife</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
           <t>Appointment Setter Jobs</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>DISBOARD-listed server functioning as an appointment-setter job board.</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>Join to view</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D84" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/server/1332654195958087681</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>General - training, networking &amp; community</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C87" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
+      <c r="D87" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>Prosper</t>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>TheCloserCommunity</t>
-        </is>
-      </c>
-      <c r="B86" s="4" t="inlineStr">
-        <is>
-          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D86" s="6" t="inlineStr">
-        <is>
-          <t>https://discord.me/8qxyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Rep</t>
-        </is>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>https://discord.me/highticketsalesrep</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Sales Pros</t>
+          <t>Prosper</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket closing skills and networking.</t>
+          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -2212,453 +2212,453 @@
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/salespros</t>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
+          <t>TheCloserCommunity</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/8qxyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>High Ticket Sales Rep</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/highticketsalesrep</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Sales Pros</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>General sales community covering high-ticket closing skills and networking.</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/salespros</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
           <t>DISBOARD - 'high-ticket-sales' tag (directory)</t>
         </is>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>Browse/discovery page listing many high-ticket-sales Discord servers, sorted by activity.</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C92" s="5" t="inlineStr">
         <is>
           <t>Directory</t>
         </is>
       </c>
-      <c r="D89" s="6" t="inlineStr">
+      <c r="D92" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="26" customHeight="1">
-      <c r="A91" s="9" t="inlineStr">
+    <row r="94" ht="26" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
         <is>
           <t>LINKEDIN</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>Job-specific - recruiters / pages posting high-ticket roles</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>Elite Closers (company page)</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>Followers vary</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
+      <c r="D97" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>High Ticket Closer Club</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>Followers vary</t>
         </is>
       </c>
-      <c r="D95" s="6" t="inlineStr">
+      <c r="D98" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>LinkedIn Jobs - 'high ticket closer / setter'</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>LinkedIn job-search feed where agencies (WFS Group, 1 Call Closers, Grant Cardone Enterprises, etc.) post high-ticket roles.</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
+      <c r="C99" s="5" t="inlineStr">
         <is>
           <t>N/A (job board)</t>
         </is>
       </c>
-      <c r="D96" s="6" t="inlineStr">
+      <c r="D99" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/search/?keywords=high%20ticket%20closer</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="2" t="inlineStr">
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>General - training pages &amp; professional community</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr">
+      <c r="C102" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D99" s="3" t="inlineStr">
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>High Ticket Sales Academy</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B103" s="4" t="inlineStr">
         <is>
           <t>Company page sharing high-ticket sales professional-development content and community.</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C103" s="5" t="inlineStr">
         <is>
           <t>Followers vary</t>
         </is>
       </c>
-      <c r="D100" s="6" t="inlineStr">
+      <c r="D103" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="4" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>Note on LinkedIn Groups</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>LinkedIn has largely sunset native 'Groups' for this niche - presence now lives in company pages, hashtags (#highticketsales, #remoteclosing) and the jobs feed.</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D101" s="5" t="inlineStr"/>
-    </row>
-    <row r="103" ht="26" customHeight="1">
-      <c r="A103" s="10" t="inlineStr">
+      <c r="D104" s="5" t="inlineStr"/>
+    </row>
+    <row r="106" ht="26" customHeight="1">
+      <c r="A106" s="10" t="inlineStr">
         <is>
           <t>CUSTOMER SUCCESS / CLIENT SUCCESS MANAGER (CSM) - ALL PLATFORMS</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="2" t="inlineStr">
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
         <is>
           <t>Job-specific - high-ticket / remote CSM training &amp; placement</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B105" s="3" t="inlineStr">
+      <c r="B108" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C105" s="3" t="inlineStr">
+      <c r="C108" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D105" s="3" t="inlineStr">
+      <c r="D108" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="4" t="inlineStr">
-        <is>
-          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
-        </is>
-      </c>
-      <c r="B106" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
-        </is>
-      </c>
-      <c r="C106" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/client-success/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="4" t="inlineStr">
-        <is>
-          <t>Client Success Club (alt)  [Skool]</t>
-        </is>
-      </c>
-      <c r="B107" s="4" t="inlineStr">
-        <is>
-          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D107" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/client-success-club/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="4" t="inlineStr">
-        <is>
-          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
-        </is>
-      </c>
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
-        </is>
-      </c>
-      <c r="C108" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/648104543815634/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
+          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/client-success/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>Client Success Club (alt)  [Skool]</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/client-success-club/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/648104543815634/</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
           <t>Virtual Assistant - Job Offers board  [Skool]</t>
         </is>
       </c>
-      <c r="B109" s="4" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>Active job board that regularly posts remote Client/Customer Success Manager openings alongside VA roles.</t>
         </is>
       </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D109" s="6" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/virtual-assistant-8842</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="2" t="inlineStr">
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>General - customer-success professional communities</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B115" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C112" s="3" t="inlineStr">
+      <c r="C115" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D112" s="3" t="inlineStr">
+      <c r="D115" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Collective  [LinkedIn + Slack]</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>10,000+ (Slack)</t>
-        </is>
-      </c>
-      <c r="D113" s="6" t="inlineStr">
-        <is>
-          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
-        </is>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>Free to join</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>https://customersuccess.network/</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>~65,000+</t>
-        </is>
-      </c>
-      <c r="D115" s="6" t="inlineStr">
-        <is>
-          <t>https://www.customersuccessassociation.com/forum/</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Leadership Network  [LinkedIn]</t>
+          <t>Customer Success Collective  [LinkedIn + Slack]</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>~14,300 followers</t>
+          <t>10,000+ (Slack)</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Gain Grow Retain  [Slack/Web]</t>
+          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
@@ -2668,58 +2668,124 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>https://gaingrowretain.com/</t>
+          <t>https://customersuccess.network/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>CS Cafe  [Slack]</t>
+          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>~65,000+</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>https://www.thecscafe.com/p/community</t>
+          <t>https://www.customersuccessassociation.com/forum/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
+          <t>Customer Success Leadership Network  [LinkedIn]</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>~14,300 followers</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>Gain Grow Retain  [Slack/Web]</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>https://gaingrowretain.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>CS Cafe  [Slack]</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thecscafe.com/p/community</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
           <t>Customer Success Network (CSM Practice)  [Facebook]</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>Facebook presence of the CS community - templates, videos, reviews and event announcements.</t>
         </is>
       </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D119" s="6" t="inlineStr">
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/customersuccessnetwork</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="70" customHeight="1">
-      <c r="A121" s="11" t="inlineStr">
-        <is>
-          <t>Notes: Member counts shown are those publicly visible at time of research (12 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
+    <row r="124" ht="70" customHeight="1">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>Notes: Member counts shown are those publicly visible at time of research (16 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
         </is>
       </c>
     </row>
@@ -2727,19 +2793,19 @@
   <mergeCells count="16">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A106:D106"/>
+    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A104:D104"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A95:D95"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A111:D111"/>
-    <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A98:D98"/>
-    <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A107:D107"/>
     <mergeCell ref="A36:D36"/>
   </mergeCells>
   <hyperlinks>
@@ -2786,7 +2852,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId47"/>
@@ -2803,30 +2869,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add The Sales Dojo (SOS Dojo) to Communities directory
</commit_message>
<xml_diff>
--- a/High_Ticket_Sales_Groups.xlsx
+++ b/High_Ticket_Sales_Groups.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2041,73 +2041,73 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="26" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>The Sales Dojo</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Premier sales-training community (SOS Dojo) with world-class training, daily coaching, a 24/7 roleplay room and connections to the best high-ticket opportunities.</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>~4,000+</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/sosdojo/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="26" customHeight="1">
+      <c r="A79" s="8" t="inlineStr">
         <is>
           <t>DISCORD</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>Job-specific - offer placement / job &amp; lead boards</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="C81" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
+      <c r="D81" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t>High Flow Closers / FlowClose</t>
-        </is>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Closers</t>
+          <t>High Flow Closers / FlowClose</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
+          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -2117,19 +2117,19 @@
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesclosers</t>
+          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Appointment Setter Life</t>
+          <t>High Ticket Sales Closers</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -2139,92 +2139,92 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/appsetterlife</t>
+          <t>https://discord.me/highticketsalesclosers</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
+          <t>Appointment Setter Life</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/appsetterlife</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
           <t>Appointment Setter Jobs</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>DISBOARD-listed server functioning as an appointment-setter job board.</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>Join to view</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr">
+      <c r="D85" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/server/1332654195958087681</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="A86" s="2" t="inlineStr">
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>General - training, networking &amp; community</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="3" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr">
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D87" s="3" t="inlineStr">
+      <c r="D88" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="4" t="inlineStr">
-        <is>
-          <t>Prosper</t>
-        </is>
-      </c>
-      <c r="B88" s="4" t="inlineStr">
-        <is>
-          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D88" s="6" t="inlineStr">
-        <is>
-          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>TheCloserCommunity</t>
+          <t>Prosper</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
+          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -2234,19 +2234,19 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/8qxyr</t>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Rep</t>
+          <t>TheCloserCommunity</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
+          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -2256,19 +2256,19 @@
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesrep</t>
+          <t>https://discord.me/8qxyr</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Sales Pros</t>
+          <t>High Ticket Sales Rep</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket closing skills and networking.</t>
+          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -2278,99 +2278,99 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/salespros</t>
+          <t>https://discord.me/highticketsalesrep</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
+          <t>Sales Pros</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>General sales community covering high-ticket closing skills and networking.</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/salespros</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
           <t>DISBOARD - 'high-ticket-sales' tag (directory)</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>Browse/discovery page listing many high-ticket-sales Discord servers, sorted by activity.</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>Directory</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="26" customHeight="1">
-      <c r="A94" s="9" t="inlineStr">
+    <row r="95" ht="26" customHeight="1">
+      <c r="A95" s="9" t="inlineStr">
         <is>
           <t>LINKEDIN</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>Job-specific - recruiters / pages posting high-ticket roles</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B97" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr">
+      <c r="C97" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D96" s="3" t="inlineStr">
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>Elite Closers (company page)</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Closer Club</t>
+          <t>Elite Closers (company page)</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
@@ -2380,168 +2380,168 @@
       </c>
       <c r="D98" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Closer Club</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn Jobs - 'high ticket closer / setter'</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>LinkedIn job-search feed where agencies (WFS Group, 1 Call Closers, Grant Cardone Enterprises, etc.) post high-ticket roles.</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>N/A (job board)</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
+      <c r="D100" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/search/?keywords=high%20ticket%20closer</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="A101" s="2" t="inlineStr">
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
         <is>
           <t>General - training pages &amp; professional community</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="3" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B103" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr">
+      <c r="C103" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D102" s="3" t="inlineStr">
+      <c r="D103" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Academy</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>Company page sharing high-ticket sales professional-development content and community.</t>
-        </is>
-      </c>
-      <c r="C103" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D103" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Sales Academy</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Company page sharing high-ticket sales professional-development content and community.</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
           <t>Note on LinkedIn Groups</t>
         </is>
       </c>
-      <c r="B104" s="4" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>LinkedIn has largely sunset native 'Groups' for this niche - presence now lives in company pages, hashtags (#highticketsales, #remoteclosing) and the jobs feed.</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C105" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr"/>
-    </row>
-    <row r="106" ht="26" customHeight="1">
-      <c r="A106" s="10" t="inlineStr">
+      <c r="D105" s="5" t="inlineStr"/>
+    </row>
+    <row r="107" ht="26" customHeight="1">
+      <c r="A107" s="10" t="inlineStr">
         <is>
           <t>CUSTOMER SUCCESS / CLIENT SUCCESS MANAGER (CSM) - ALL PLATFORMS</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="A107" s="2" t="inlineStr">
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
         <is>
           <t>Job-specific - high-ticket / remote CSM training &amp; placement</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="3" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C108" s="3" t="inlineStr">
+      <c r="C109" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D108" s="3" t="inlineStr">
+      <c r="D109" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="4" t="inlineStr">
-        <is>
-          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
-        </is>
-      </c>
-      <c r="B109" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
-        </is>
-      </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Client Success Club (alt)  [Skool]</t>
+          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
+          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
@@ -2551,19 +2551,19 @@
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/client-success-club/about</t>
+          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+          <t>Client Success Club (alt)  [Skool]</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
@@ -2573,180 +2573,180 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/648104543815634/</t>
+          <t>https://www.skool.com/client-success-club/about</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
+          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/648104543815634/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
           <t>Virtual Assistant - Job Offers board  [Skool]</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>Active job board that regularly posts remote Client/Customer Success Manager openings alongside VA roles.</t>
         </is>
       </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/virtual-assistant-8842</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="2" t="inlineStr">
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>General - customer-success professional communities</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="3" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B116" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C115" s="3" t="inlineStr">
+      <c r="C116" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D115" s="3" t="inlineStr">
+      <c r="D116" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Collective  [LinkedIn + Slack]</t>
-        </is>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>10,000+ (Slack)</t>
-        </is>
-      </c>
-      <c r="D116" s="6" t="inlineStr">
-        <is>
-          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
+          <t>Customer Success Collective  [LinkedIn + Slack]</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
+          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>10,000+ (Slack)</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>https://customersuccess.network/</t>
+          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
+          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
+          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>~65,000+</t>
+          <t>Free to join</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>https://www.customersuccessassociation.com/forum/</t>
+          <t>https://customersuccess.network/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Leadership Network  [LinkedIn]</t>
+          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>~14,300 followers</t>
+          <t>~65,000+</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+          <t>https://www.customersuccessassociation.com/forum/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Gain Grow Retain  [Slack/Web]</t>
+          <t>Customer Success Leadership Network  [LinkedIn]</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>~14,300 followers</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>https://gaingrowretain.com/</t>
+          <t>https://www.linkedin.com/company/cs-leadership-network</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>CS Cafe  [Slack]</t>
+          <t>Gain Grow Retain  [Slack/Web]</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
@@ -2756,34 +2756,56 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>https://www.thecscafe.com/p/community</t>
+          <t>https://gaingrowretain.com/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
+          <t>CS Cafe  [Slack]</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thecscafe.com/p/community</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
           <t>Customer Success Network (CSM Practice)  [Facebook]</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B123" s="4" t="inlineStr">
         <is>
           <t>Facebook presence of the CS community - templates, videos, reviews and event announcements.</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D122" s="6" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/customersuccessnetwork</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="70" customHeight="1">
-      <c r="A124" s="11" t="inlineStr">
+    <row r="125" ht="70" customHeight="1">
+      <c r="A125" s="11" t="inlineStr">
         <is>
           <t>Notes: Member counts shown are those publicly visible at time of research (16 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
         </is>
@@ -2791,21 +2813,21 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A102:D102"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A106:D106"/>
-    <mergeCell ref="A114:D114"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A108:D108"/>
     <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A124:D124"/>
-    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A87:D87"/>
     <mergeCell ref="A95:D95"/>
+    <mergeCell ref="A125:D125"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A107:D107"/>
+    <mergeCell ref="A115:D115"/>
     <mergeCell ref="A36:D36"/>
   </mergeCells>
   <hyperlinks>
@@ -2872,30 +2894,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add The Game of Influence to Skool communities; keep analytics in directory template
Add The Game of Influence (Skool) to the general training/community list and
regenerate the directory (90 communities). Also bake the Vercel + GoatCounter
analytics snippets into build.py's template so regenerating the directory no
longer wipes the tracking tags.

https://claude.ai/code/session_01GUJ8qSByy4U4SPUEowsMsA
</commit_message>
<xml_diff>
--- a/High_Ticket_Sales_Groups.xlsx
+++ b/High_Ticket_Sales_Groups.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2063,73 +2063,73 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="8" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>The Game of Influence</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Mentor-led high-ticket sales community focused on turning members into remote closers earning $10k+/mo, pairing training and mentorship with job opportunities.</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skool.com/the-game-of-influence/about</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="26" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>DISCORD</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>Job-specific - offer placement / job &amp; lead boards</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="inlineStr">
-        <is>
-          <t>High Flow Closers / FlowClose</t>
-        </is>
-      </c>
-      <c r="B82" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Closers</t>
+          <t>High Flow Closers / FlowClose</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
+          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -2139,19 +2139,19 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesclosers</t>
+          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Appointment Setter Life</t>
+          <t>High Ticket Sales Closers</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -2161,92 +2161,92 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/appsetterlife</t>
+          <t>https://discord.me/highticketsalesclosers</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
+          <t>Appointment Setter Life</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/appsetterlife</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
           <t>Appointment Setter Jobs</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>DISBOARD-listed server functioning as an appointment-setter job board.</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>Join to view</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/server/1332654195958087681</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>General - training, networking &amp; community</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
+      <c r="D89" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="4" t="inlineStr">
-        <is>
-          <t>Prosper</t>
-        </is>
-      </c>
-      <c r="B89" s="4" t="inlineStr">
-        <is>
-          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>TheCloserCommunity</t>
+          <t>Prosper</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
+          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -2256,19 +2256,19 @@
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/8qxyr</t>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Rep</t>
+          <t>TheCloserCommunity</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
+          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -2278,19 +2278,19 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesrep</t>
+          <t>https://discord.me/8qxyr</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Sales Pros</t>
+          <t>High Ticket Sales Rep</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket closing skills and networking.</t>
+          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -2300,99 +2300,99 @@
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/salespros</t>
+          <t>https://discord.me/highticketsalesrep</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
+          <t>Sales Pros</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>General sales community covering high-ticket closing skills and networking.</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/salespros</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
           <t>DISBOARD - 'high-ticket-sales' tag (directory)</t>
         </is>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>Browse/discovery page listing many high-ticket-sales Discord servers, sorted by activity.</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>Directory</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D94" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="26" customHeight="1">
-      <c r="A95" s="9" t="inlineStr">
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
         <is>
           <t>LINKEDIN</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="2" t="inlineStr">
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>Job-specific - recruiters / pages posting high-ticket roles</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C97" s="3" t="inlineStr">
+      <c r="C98" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D97" s="3" t="inlineStr">
+      <c r="D98" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>Elite Closers (company page)</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Closer Club</t>
+          <t>Elite Closers (company page)</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -2402,168 +2402,168 @@
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Closer Club</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn Jobs - 'high ticket closer / setter'</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>LinkedIn job-search feed where agencies (WFS Group, 1 Call Closers, Grant Cardone Enterprises, etc.) post high-ticket roles.</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C101" s="5" t="inlineStr">
         <is>
           <t>N/A (job board)</t>
         </is>
       </c>
-      <c r="D100" s="6" t="inlineStr">
+      <c r="D101" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/search/?keywords=high%20ticket%20closer</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="2" t="inlineStr">
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>General - training pages &amp; professional community</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C104" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D103" s="3" t="inlineStr">
+      <c r="D104" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Academy</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>Company page sharing high-ticket sales professional-development content and community.</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Sales Academy</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Company page sharing high-ticket sales professional-development content and community.</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
           <t>Note on LinkedIn Groups</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>LinkedIn has largely sunset native 'Groups' for this niche - presence now lives in company pages, hashtags (#highticketsales, #remoteclosing) and the jobs feed.</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr"/>
-    </row>
-    <row r="107" ht="26" customHeight="1">
-      <c r="A107" s="10" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr"/>
+    </row>
+    <row r="108" ht="26" customHeight="1">
+      <c r="A108" s="10" t="inlineStr">
         <is>
           <t>CUSTOMER SUCCESS / CLIENT SUCCESS MANAGER (CSM) - ALL PLATFORMS</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="2" t="inlineStr">
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>Job-specific - high-ticket / remote CSM training &amp; placement</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C109" s="3" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D109" s="3" t="inlineStr">
+      <c r="D110" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="4" t="inlineStr">
-        <is>
-          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
-        </is>
-      </c>
-      <c r="B110" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
-        </is>
-      </c>
-      <c r="C110" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Client Success Club (alt)  [Skool]</t>
+          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
+          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
@@ -2573,19 +2573,19 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/client-success-club/about</t>
+          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+          <t>Client Success Club (alt)  [Skool]</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -2595,180 +2595,180 @@
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/648104543815634/</t>
+          <t>https://www.skool.com/client-success-club/about</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
+          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/648104543815634/</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
           <t>Virtual Assistant - Job Offers board  [Skool]</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>Active job board that regularly posts remote Client/Customer Success Manager openings alongside VA roles.</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D113" s="6" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/virtual-assistant-8842</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="2" t="inlineStr">
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>General - customer-success professional communities</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="3" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B117" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C116" s="3" t="inlineStr">
+      <c r="C117" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D116" s="3" t="inlineStr">
+      <c r="D117" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Collective  [LinkedIn + Slack]</t>
-        </is>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
-        </is>
-      </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>10,000+ (Slack)</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
+          <t>Customer Success Collective  [LinkedIn + Slack]</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
+          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>10,000+ (Slack)</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>https://customersuccess.network/</t>
+          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
+          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
+          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>~65,000+</t>
+          <t>Free to join</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>https://www.customersuccessassociation.com/forum/</t>
+          <t>https://customersuccess.network/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Leadership Network  [LinkedIn]</t>
+          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>~14,300 followers</t>
+          <t>~65,000+</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+          <t>https://www.customersuccessassociation.com/forum/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Gain Grow Retain  [Slack/Web]</t>
+          <t>Customer Success Leadership Network  [LinkedIn]</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>~14,300 followers</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>https://gaingrowretain.com/</t>
+          <t>https://www.linkedin.com/company/cs-leadership-network</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>CS Cafe  [Slack]</t>
+          <t>Gain Grow Retain  [Slack/Web]</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -2778,34 +2778,56 @@
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>https://www.thecscafe.com/p/community</t>
+          <t>https://gaingrowretain.com/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
+          <t>CS Cafe  [Slack]</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thecscafe.com/p/community</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
           <t>Customer Success Network (CSM Practice)  [Facebook]</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>Facebook presence of the CS community - templates, videos, reviews and event announcements.</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D123" s="6" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/customersuccessnetwork</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="70" customHeight="1">
-      <c r="A125" s="11" t="inlineStr">
+    <row r="126" ht="70" customHeight="1">
+      <c r="A126" s="11" t="inlineStr">
         <is>
           <t>Notes: Member counts shown are those publicly visible at time of research (16 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
         </is>
@@ -2813,21 +2835,21 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A102:D102"/>
+    <mergeCell ref="A116:D116"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A79:D79"/>
     <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A103:D103"/>
     <mergeCell ref="A108:D108"/>
+    <mergeCell ref="A126:D126"/>
+    <mergeCell ref="A88:D88"/>
+    <mergeCell ref="A97:D97"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A125:D125"/>
+    <mergeCell ref="A109:D109"/>
+    <mergeCell ref="A81:D81"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A107:D107"/>
-    <mergeCell ref="A115:D115"/>
     <mergeCell ref="A36:D36"/>
   </mergeCells>
   <hyperlinks>
@@ -2895,30 +2917,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Separate The Sales Dojo (Sensei CJ) from SOS Dojo; use real listing data
These are two different communities. Restore the SOS Dojo entry to its own
skool.com/sosdojo URL (renamed 'The Sales Dojo (SOS Dojo)'), and add the
correct The Sales Dojo (Sensei CJ, skool.com/sales-dojo) as its own entry +
the premium spotlight, with accurate copy (black-belt closer training, ~19
members, $172/mo) and the referral link.

https://claude.ai/code/session_01GUJ8qSByy4U4SPUEowsMsA
</commit_message>
<xml_diff>
--- a/High_Ticket_Sales_Groups.xlsx
+++ b/High_Ticket_Sales_Groups.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2044,12 +2044,12 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>The Sales Dojo</t>
+          <t>The Sales Dojo (SOS Dojo)</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Premier sales-training community (SOS Dojo) with world-class training, daily coaching, a 24/7 roleplay room and connections to the best high-ticket opportunities.</t>
+          <t>Sales-training community (SOS Dojo) with world-class training, daily coaching, a 24/7 roleplay room and connections to the best high-ticket opportunities.</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -2059,99 +2059,99 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>http://www.skool.com/sales-dojo?utm_campaign=skool_link_post&amp;utm_content=96652a20bde64d799137b6c75716a2de</t>
+          <t>https://www.skool.com/sosdojo/about</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
+          <t>The Sales Dojo</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Sensei CJ's high-ticket sales 'dojo' — train hard to become a 'black belt' closer who gets paid consistently, through daily study, live coaching, call reviews, number tracking and identity work. Earn your investment back inside. $172/mo.</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>~19</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>http://www.skool.com/sales-dojo?utm_campaign=skool_link_post&amp;utm_content=96652a20bde64d799137b6c75716a2de</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
           <t>The Game of Influence</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>Mentor-led high-ticket sales community focused on turning members into remote closers earning $10k+/mo, pairing training and mentorship with job opportunities.</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/the-game-of-influence/about</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="8" t="inlineStr">
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="8" t="inlineStr">
         <is>
           <t>DISCORD</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="2" t="inlineStr">
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Job-specific - offer placement / job &amp; lead boards</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C83" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>High Flow Closers / FlowClose</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Closers</t>
+          <t>High Flow Closers / FlowClose</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
+          <t>Bills itself as the #1 sales &amp; offer-placement community - free offer placements, scripts, networking and weekly giveaways for closers/setters.</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -2161,19 +2161,19 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesclosers</t>
+          <t>https://top.gg/discord/servers/766313238700785664</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Appointment Setter Life</t>
+          <t>High Ticket Sales Closers</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+          <t>Offers ~20,000 free email/phone leads per month, free high-ticket courses, networking and webinars.</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -2183,92 +2183,92 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/appsetterlife</t>
+          <t>https://discord.me/highticketsalesclosers</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
+          <t>Appointment Setter Life</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Setter-focused server with free leads and high-ticket content for setters/closers.</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/appsetterlife</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
           <t>Appointment Setter Jobs</t>
         </is>
       </c>
-      <c r="B86" s="4" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>DISBOARD-listed server functioning as an appointment-setter job board.</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>Join to view</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/server/1332654195958087681</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>General - training, networking &amp; community</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="3" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B90" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C89" s="3" t="inlineStr">
+      <c r="C90" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D89" s="3" t="inlineStr">
+      <c r="D90" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="inlineStr">
-        <is>
-          <t>Prosper</t>
-        </is>
-      </c>
-      <c r="B90" s="4" t="inlineStr">
-        <is>
-          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>Join to view</t>
-        </is>
-      </c>
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>TheCloserCommunity</t>
+          <t>Prosper</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
+          <t>Results-driven community for mastering high-ticket sales and scaling income - frameworks, closing, client acquisition, personal branding.</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -2278,19 +2278,19 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/8qxyr</t>
+          <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Sales Rep</t>
+          <t>TheCloserCommunity</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
+          <t>100% free community where high-ticket closers motivate each other to close more deals; shares leads and courses.</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -2300,19 +2300,19 @@
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/highticketsalesrep</t>
+          <t>https://discord.me/8qxyr</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Sales Pros</t>
+          <t>High Ticket Sales Rep</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>General sales community covering high-ticket closing skills and networking.</t>
+          <t>Server for high-ticket sales reps - free leads, courses and networking.</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -2322,99 +2322,99 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>https://discord.me/salespros</t>
+          <t>https://discord.me/highticketsalesrep</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
+          <t>Sales Pros</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>General sales community covering high-ticket closing skills and networking.</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Join to view</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>https://discord.me/salespros</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
           <t>DISBOARD - 'high-ticket-sales' tag (directory)</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>Browse/discovery page listing many high-ticket-sales Discord servers, sorted by activity.</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C95" s="5" t="inlineStr">
         <is>
           <t>Directory</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
+      <c r="D95" s="6" t="inlineStr">
         <is>
           <t>https://disboard.org/servers/tag/high-ticket-sales</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="26" customHeight="1">
-      <c r="A96" s="9" t="inlineStr">
+    <row r="97" ht="26" customHeight="1">
+      <c r="A97" s="9" t="inlineStr">
         <is>
           <t>LINKEDIN</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="20" customHeight="1">
-      <c r="A97" s="2" t="inlineStr">
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>Job-specific - recruiters / pages posting high-ticket roles</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="3" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C98" s="3" t="inlineStr">
+      <c r="C99" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D98" s="3" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>Elite Closers (company page)</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
-        </is>
-      </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>High Ticket Closer Club</t>
+          <t>Elite Closers (company page)</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+          <t>High-ticket sales company connecting the top 1% of business owners with top 1% sales professionals; posts roles.</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -2424,168 +2424,168 @@
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+          <t>https://www.linkedin.com/company/eliteclosers</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Closer Club</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Invitation-only sales-training/opportunity built around Grant Cardone content for closers raising their income.</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-closer-club</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn Jobs - 'high ticket closer / setter'</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>LinkedIn job-search feed where agencies (WFS Group, 1 Call Closers, Grant Cardone Enterprises, etc.) post high-ticket roles.</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C102" s="5" t="inlineStr">
         <is>
           <t>N/A (job board)</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D102" s="6" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/search/?keywords=high%20ticket%20closer</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="20" customHeight="1">
-      <c r="A103" s="2" t="inlineStr">
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>General - training pages &amp; professional community</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="B105" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C104" s="3" t="inlineStr">
+      <c r="C105" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D104" s="3" t="inlineStr">
+      <c r="D105" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
-        <is>
-          <t>High Ticket Sales Academy</t>
-        </is>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t>Company page sharing high-ticket sales professional-development content and community.</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>Followers vary</t>
-        </is>
-      </c>
-      <c r="D105" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
+          <t>High Ticket Sales Academy</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Company page sharing high-ticket sales professional-development content and community.</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Followers vary</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/high-ticket-sales-academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
           <t>Note on LinkedIn Groups</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>LinkedIn has largely sunset native 'Groups' for this niche - presence now lives in company pages, hashtags (#highticketsales, #remoteclosing) and the jobs feed.</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C107" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D106" s="5" t="inlineStr"/>
-    </row>
-    <row r="108" ht="26" customHeight="1">
-      <c r="A108" s="10" t="inlineStr">
+      <c r="D107" s="5" t="inlineStr"/>
+    </row>
+    <row r="109" ht="26" customHeight="1">
+      <c r="A109" s="10" t="inlineStr">
         <is>
           <t>CUSTOMER SUCCESS / CLIENT SUCCESS MANAGER (CSM) - ALL PLATFORMS</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="A109" s="2" t="inlineStr">
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>Job-specific - high-ticket / remote CSM training &amp; placement</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="3" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D110" s="3" t="inlineStr">
+      <c r="D111" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
-        <is>
-          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
-        </is>
-      </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D111" s="6" t="inlineStr">
-        <is>
-          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Client Success Club (alt)  [Skool]</t>
+          <t>Client Success Club (CSC) - Robert Lyon  [Skool]</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
+          <t>Bills itself as the #1 community for landing high-paying remote CSM roles ($10k-25k/mo) for high-ticket businesses; training, job board, weekly coaching.</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -2595,19 +2595,19 @@
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>https://www.skool.com/client-success-club/about</t>
+          <t>https://www.skool.com/client-success/about</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+          <t>Client Success Club (alt)  [Skool]</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+          <t>Client-success-manager training &amp; community focused on landing remote high-ticket CSM roles.</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
@@ -2617,180 +2617,180 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/648104543815634/</t>
+          <t>https://www.skool.com/client-success-club/about</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
+          <t>Remote Sales / CSM Jobs (Sales Pipeline Pros - Group #3)  [Facebook]</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Facebook job board posting remote sales AND customer/client success manager roles.</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/648104543815634/</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
           <t>Virtual Assistant - Job Offers board  [Skool]</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>Active job board that regularly posts remote Client/Customer Success Manager openings alongside VA roles.</t>
         </is>
       </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>https://www.skool.com/virtual-assistant-8842</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="2" t="inlineStr">
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>General - customer-success professional communities</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="3" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
         <is>
           <t>Group / Community</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B118" s="3" t="inlineStr">
         <is>
           <t>What it's advertised as</t>
         </is>
       </c>
-      <c r="C117" s="3" t="inlineStr">
+      <c r="C118" s="3" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
-      <c r="D117" s="3" t="inlineStr">
+      <c r="D118" s="3" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Collective  [LinkedIn + Slack]</t>
-        </is>
-      </c>
-      <c r="B118" s="4" t="inlineStr">
-        <is>
-          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
-        </is>
-      </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>10,000+ (Slack)</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
+          <t>Customer Success Collective  [LinkedIn + Slack]</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
+          <t>Global CS community (junior CSM to CCO) with a 10,000+ member Slack, templates, articles, events and job board.</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>10,000+ (Slack)</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>https://customersuccess.network/</t>
+          <t>https://www.customersuccesscollective.com/customer-success-community/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
+          <t>Customer Success Network (CSN)  [LinkedIn + Workplace]</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
+          <t>First global peer-learning CS community; free access to an online community to ask questions and network with CSMs/CS leaders.</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>~65,000+</t>
+          <t>Free to join</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>https://www.customersuccessassociation.com/forum/</t>
+          <t>https://customersuccess.network/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Customer Success Leadership Network  [LinkedIn]</t>
+          <t>The Customer Success Forum (CS Association)  [Web/LinkedIn]</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
+          <t>Long-running professional discussion forum spanning CEOs to practising CSMs across all company sizes worldwide.</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>~14,300 followers</t>
+          <t>~65,000+</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/cs-leadership-network</t>
+          <t>https://www.customersuccessassociation.com/forum/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>Gain Grow Retain  [Slack/Web]</t>
+          <t>Customer Success Leadership Network  [LinkedIn]</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
+          <t>Content + connection network focused on sustaining the CS function and CS leadership.</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Free to join</t>
+          <t>~14,300 followers</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>https://gaingrowretain.com/</t>
+          <t>https://www.linkedin.com/company/cs-leadership-network</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>CS Cafe  [Slack]</t>
+          <t>Gain Grow Retain  [Slack/Web]</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+          <t>Peer-to-peer community for B2B SaaS customer-success leaders - team structure, retention, cross-collaboration.</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
@@ -2800,34 +2800,56 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>https://www.thecscafe.com/p/community</t>
+          <t>https://gaingrowretain.com/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
+          <t>CS Cafe  [Slack]</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Slack network for customer-success professionals to connect, share and find roles.</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Free to join</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thecscafe.com/p/community</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
           <t>Customer Success Network (CSM Practice)  [Facebook]</t>
         </is>
       </c>
-      <c r="B124" s="4" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>Facebook presence of the CS community - templates, videos, reviews and event announcements.</t>
         </is>
       </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>Login required</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Login required</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/customersuccessnetwork</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="70" customHeight="1">
-      <c r="A126" s="11" t="inlineStr">
+    <row r="127" ht="70" customHeight="1">
+      <c r="A127" s="11" t="inlineStr">
         <is>
           <t>Notes: Member counts shown are those publicly visible at time of research (16 Jun 2026). 'Login required' / 'Join to view' means the platform hides the count behind a login. Discord servers are reached via invite/listing pages and counts fluctuate. LinkedIn has largely retired native Groups for this niche, so its presence is company pages + the jobs feed. CSM rows are tagged with their platform in [brackets]. Many of these are marketing/lead-gen communities for paid programs - verify before outreach.</t>
         </is>
@@ -2835,21 +2857,21 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A116:D116"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A108:D108"/>
-    <mergeCell ref="A126:D126"/>
-    <mergeCell ref="A88:D88"/>
+    <mergeCell ref="A110:D110"/>
+    <mergeCell ref="A89:D89"/>
     <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A127:D127"/>
     <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A96:D96"/>
     <mergeCell ref="A109:D109"/>
+    <mergeCell ref="A104:D104"/>
+    <mergeCell ref="A82:D82"/>
     <mergeCell ref="A81:D81"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A98:D98"/>
     <mergeCell ref="A36:D36"/>
   </mergeCells>
   <hyperlinks>
@@ -2918,30 +2940,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>